<commit_message>
Sync from job_collector-private (scrubbed)
Automated publish via scripts/sync_public_repo.py.
</commit_message>
<xml_diff>
--- a/data/processed/crypto_jobs_clean_v1.xlsx
+++ b/data/processed/crypto_jobs_clean_v1.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="jobs_master" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="jobs_view" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="jobs_text" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="manual_review" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="active_near_fit" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="applications" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="skills_gap" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="skill_recommendations" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="jobs_master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="jobs_view" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="jobs_text" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="manual_review" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="applications" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skills_gap" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skill_recommendations" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="active_near_fit" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1083,90 +1083,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>decision</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>city_region</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>work_mode</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>seniority_manual</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>main_reason</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>review_notes</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1233,7 +1149,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1271,7 +1187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1341,4 +1257,88 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>city_region</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>work_mode</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>seniority_manual</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>main_reason</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>review_notes</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>